<commit_message>
Introduction masse généralisée par TMN dans DLL_CTICM_MODAL
</commit_message>
<xml_diff>
--- a/VALIDATION/CAS F06/Cas F06.xlsx
+++ b/VALIDATION/CAS F06/Cas F06.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\RAID 1\LOGICIELS\CTICM AM - POUTRE MIXTE\DEV23\VALIDATION\CAS F06\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A1B212D-D1F6-464B-B554-1BCD10C10E72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08EAC788-B347-4C40-B1B7-0DFDB9D89F81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1B2E1AE3-11FD-420F-B8DC-6BB03E477683}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{1B2E1AE3-11FD-420F-B8DC-6BB03E477683}"/>
   </bookViews>
   <sheets>
     <sheet name="Données" sheetId="1" r:id="rId1"/>
@@ -50,9 +50,11 @@
     <definedName name="krmin">Données!$O$20</definedName>
     <definedName name="LL">Données!$E$23</definedName>
     <definedName name="Massiv">Données!$O$16</definedName>
+    <definedName name="MEd">Données!$E$26</definedName>
     <definedName name="nbPhi">Données!$O$10</definedName>
     <definedName name="p">Données!$E$59</definedName>
     <definedName name="Phi">Données!$O$9</definedName>
+    <definedName name="qELU">Données!$E$24</definedName>
     <definedName name="Rr">Données!$J$11</definedName>
     <definedName name="tcp">Données!$E$60</definedName>
     <definedName name="Td">Données!$E$8</definedName>
@@ -61,6 +63,7 @@
     <definedName name="u">Données!$O$23</definedName>
     <definedName name="ui">Données!$O$11</definedName>
     <definedName name="usi">Données!$O$12</definedName>
+    <definedName name="VEd">Données!$E$27</definedName>
     <definedName name="zANP">Données!$E$61</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -106,7 +109,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="86">
   <si>
     <t>Dalle</t>
   </si>
@@ -340,6 +343,30 @@
   </si>
   <si>
     <t>zA</t>
+  </si>
+  <si>
+    <t>zsinf</t>
+  </si>
+  <si>
+    <t>Charge</t>
+  </si>
+  <si>
+    <t>kN/m</t>
+  </si>
+  <si>
+    <t>Moment maxi</t>
+  </si>
+  <si>
+    <t>V maxi</t>
+  </si>
+  <si>
+    <t>Critères</t>
+  </si>
+  <si>
+    <t>GammaM</t>
+  </si>
+  <si>
+    <t>GammaV</t>
   </si>
 </sst>
 </file>
@@ -377,7 +404,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -420,8 +447,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -493,6 +526,15 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
@@ -505,11 +547,71 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -556,6 +658,9 @@
     <xf numFmtId="167" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -587,7 +692,22 @@
     <xf numFmtId="168" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="8" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="11" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="12" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -930,23 +1050,59 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B56F61FB-A83D-4407-8208-02CCB2B8B274}">
-  <dimension ref="B2:T75"/>
+  <dimension ref="B2:T81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D2" t="s">
+      <c r="D2" s="31" t="s">
         <v>15</v>
       </c>
+      <c r="E2" s="32"/>
+      <c r="F2" s="32"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="32"/>
+      <c r="I2" s="32"/>
+      <c r="J2" s="32"/>
+      <c r="K2" s="32"/>
+      <c r="L2" s="32"/>
+      <c r="M2" s="32"/>
+      <c r="N2" s="32"/>
+      <c r="O2" s="32"/>
+      <c r="P2" s="33"/>
     </row>
     <row r="3" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D3" t="s">
+      <c r="D3" s="34" t="s">
         <v>16</v>
       </c>
+      <c r="E3" s="35"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="35"/>
+      <c r="H3" s="35"/>
+      <c r="I3" s="35"/>
+      <c r="J3" s="35"/>
+      <c r="K3" s="35"/>
+      <c r="L3" s="35"/>
+      <c r="M3" s="35"/>
+      <c r="N3" s="35"/>
+      <c r="O3" s="35"/>
+      <c r="P3" s="36"/>
     </row>
     <row r="4" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D4" t="s">
+      <c r="D4" s="37" t="s">
         <v>17</v>
       </c>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
+      <c r="G4" s="38"/>
+      <c r="H4" s="38"/>
+      <c r="I4" s="38"/>
+      <c r="J4" s="38"/>
+      <c r="K4" s="38"/>
+      <c r="L4" s="38"/>
+      <c r="M4" s="38"/>
+      <c r="N4" s="38"/>
+      <c r="O4" s="38"/>
+      <c r="P4" s="39"/>
     </row>
     <row r="6" spans="4:16" x14ac:dyDescent="0.25">
       <c r="D6" s="1" t="s">
@@ -1062,7 +1218,7 @@
         <v>6</v>
       </c>
       <c r="E11" s="6">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F11" t="s">
         <v>4</v>
@@ -1136,7 +1292,7 @@
       </c>
       <c r="E14" s="10">
         <f>(Td-hp)-hcfi</f>
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F14" t="s">
         <v>4</v>
@@ -1341,6 +1497,15 @@
       </c>
     </row>
     <row r="24" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D24" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E24" s="6">
+        <v>20</v>
+      </c>
+      <c r="F24" t="s">
+        <v>80</v>
+      </c>
       <c r="J24" s="4"/>
       <c r="N24" s="3"/>
       <c r="O24" s="4"/>
@@ -1360,11 +1525,24 @@
         <v>67</v>
       </c>
       <c r="O25" s="15">
-        <f>MIN(krmax,MAX(krmin,(u*a_3+a_4)*a_5/SQRT(Massiv)))</f>
+        <f>O26</f>
         <v>0.39514579958198603</v>
       </c>
+      <c r="P25">
+        <v>0.435</v>
+      </c>
     </row>
     <row r="26" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D26" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="E26" s="14">
+        <f>qELU*LL^2/8</f>
+        <v>390.625</v>
+      </c>
+      <c r="F26" t="s">
+        <v>74</v>
+      </c>
       <c r="I26" s="11" t="s">
         <v>28</v>
       </c>
@@ -1376,9 +1554,22 @@
         <v>4</v>
       </c>
       <c r="N26" s="3"/>
-      <c r="O26" s="4"/>
+      <c r="O26" s="15">
+        <f>MIN(krmax,MAX(krmin,(u*a_3+a_4)*a_5/SQRT(Massiv)))</f>
+        <v>0.39514579958198603</v>
+      </c>
     </row>
     <row r="27" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D27" s="11" t="s">
+        <v>82</v>
+      </c>
+      <c r="E27" s="10">
+        <f>qELU*LL/2</f>
+        <v>125</v>
+      </c>
+      <c r="F27" t="s">
+        <v>44</v>
+      </c>
       <c r="I27" s="11" t="s">
         <v>29</v>
       </c>
@@ -1436,7 +1627,7 @@
       </c>
       <c r="N32" s="3"/>
     </row>
-    <row r="33" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:16" x14ac:dyDescent="0.25">
       <c r="I33" s="11" t="s">
         <v>35</v>
       </c>
@@ -1446,7 +1637,7 @@
       </c>
       <c r="N33" s="3"/>
     </row>
-    <row r="36" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:16" x14ac:dyDescent="0.25">
       <c r="E36" s="5" t="s">
         <v>24</v>
       </c>
@@ -1459,32 +1650,44 @@
       <c r="H36" s="5" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="37" spans="2:14" x14ac:dyDescent="0.25">
-      <c r="E37" s="18" t="s">
+      <c r="N36" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+    </row>
+    <row r="37" spans="2:16" x14ac:dyDescent="0.25">
+      <c r="E37" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="F37" s="18" t="s">
+      <c r="F37" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="G37" s="18" t="s">
+      <c r="G37" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="H37" s="18" t="s">
+      <c r="H37" s="19" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="38" spans="2:14" x14ac:dyDescent="0.25">
+      <c r="N37" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="O37" s="41">
+        <f>MEd/I75</f>
+        <v>0.62402482897499145</v>
+      </c>
+    </row>
+    <row r="38" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D38" s="3" t="s">
         <v>37</v>
       </c>
       <c r="E38" s="5">
         <f>hch*beff*1000</f>
-        <v>127500</v>
+        <v>130000</v>
       </c>
       <c r="F38" s="5">
         <f>Ht+Td-hch/2</f>
-        <v>611.5</v>
+        <v>611</v>
       </c>
       <c r="G38" s="13">
         <f>fck/GammaC</f>
@@ -1492,18 +1695,22 @@
       </c>
       <c r="H38" s="13">
         <f>G38*E38/1000</f>
-        <v>2942.3076923076924</v>
-      </c>
-      <c r="I38" s="21">
+        <v>3000</v>
+      </c>
+      <c r="I38" s="22">
         <f>H38</f>
-        <v>2942.3076923076924</v>
-      </c>
-      <c r="J38" s="21">
+        <v>3000</v>
+      </c>
+      <c r="J38" s="22">
         <f t="shared" ref="J38:J52" si="0">J39+H38</f>
-        <v>5163.5331792633115</v>
-      </c>
-    </row>
-    <row r="39" spans="2:14" x14ac:dyDescent="0.25">
+        <v>5221.2254869556182</v>
+      </c>
+      <c r="N38" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="O38" s="40"/>
+    </row>
+    <row r="39" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D39" s="3" t="s">
         <v>38</v>
       </c>
@@ -1513,30 +1720,30 @@
       </c>
       <c r="F39" s="5">
         <f>Ht+Td-hch-hcfi/2</f>
-        <v>571</v>
+        <v>570</v>
       </c>
       <c r="G39" s="13">
         <f>fck/GammaC</f>
         <v>23.076923076923077</v>
       </c>
-      <c r="H39" s="19">
+      <c r="H39" s="20">
         <f t="shared" ref="H39:H54" si="1">G39*E39/1000</f>
         <v>138.46153846153848</v>
       </c>
-      <c r="I39" s="21">
+      <c r="I39" s="22">
         <f>I38+H39</f>
-        <v>3080.7692307692309</v>
-      </c>
-      <c r="J39" s="21">
+        <v>3138.4615384615386</v>
+      </c>
+      <c r="J39" s="22">
         <f t="shared" si="0"/>
         <v>2221.2254869556186</v>
       </c>
     </row>
-    <row r="40" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D40" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E40" s="19">
+      <c r="E40" s="20">
         <f>Tf*(bf-2*dbfi)</f>
         <v>1819.75</v>
       </c>
@@ -1548,20 +1755,20 @@
         <f>fy/gammaM</f>
         <v>355</v>
       </c>
-      <c r="H40" s="19">
+      <c r="H40" s="20">
         <f t="shared" si="1"/>
         <v>646.01125000000002</v>
       </c>
-      <c r="I40" s="21">
+      <c r="I40" s="22">
         <f t="shared" ref="I40:I54" si="2">I39+H40</f>
-        <v>3726.780480769231</v>
-      </c>
-      <c r="J40" s="21">
+        <v>3784.4727884615386</v>
+      </c>
+      <c r="J40" s="22">
         <f t="shared" si="0"/>
         <v>2082.7639484940801</v>
       </c>
     </row>
-    <row r="41" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D41" s="3" t="s">
         <v>49</v>
       </c>
@@ -1569,29 +1776,29 @@
         <f>(4-PI())*Rr^2/2+Rr*Tw</f>
         <v>0</v>
       </c>
-      <c r="F41" s="23"/>
+      <c r="F41" s="24"/>
       <c r="G41" s="5">
         <f>fy/gammaM</f>
         <v>355</v>
       </c>
-      <c r="H41" s="22">
+      <c r="H41" s="23">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="I41" s="21">
+      <c r="I41" s="22">
         <f t="shared" si="2"/>
-        <v>3726.780480769231</v>
-      </c>
-      <c r="J41" s="21">
+        <v>3784.4727884615386</v>
+      </c>
+      <c r="J41" s="22">
         <f t="shared" si="0"/>
         <v>1436.7526984940801</v>
       </c>
     </row>
-    <row r="42" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:16" x14ac:dyDescent="0.25">
       <c r="D42" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E42" s="19">
+      <c r="E42" s="20">
         <f>(hh-Rr)*Tw</f>
         <v>3289.9605633802817</v>
       </c>
@@ -1603,20 +1810,20 @@
         <f>G41</f>
         <v>355</v>
       </c>
-      <c r="H42" s="22">
+      <c r="H42" s="23">
         <f t="shared" si="1"/>
         <v>1167.9359999999999</v>
       </c>
-      <c r="I42" s="21">
+      <c r="I42" s="22">
         <f t="shared" si="2"/>
-        <v>4894.7164807692307</v>
-      </c>
-      <c r="J42" s="21">
+        <v>4952.4087884615383</v>
+      </c>
+      <c r="J42" s="22">
         <f t="shared" si="0"/>
         <v>1436.7526984940801</v>
       </c>
     </row>
-    <row r="43" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:16" x14ac:dyDescent="0.25">
       <c r="B43" s="3" t="s">
         <v>51</v>
       </c>
@@ -1627,11 +1834,11 @@
       <c r="D43" s="3">
         <v>1</v>
       </c>
-      <c r="E43" s="20">
+      <c r="E43" s="21">
         <f>(hl/10)*Tw</f>
         <v>64.123943661971836</v>
       </c>
-      <c r="F43" s="20">
+      <c r="F43" s="21">
         <f>Tf+hl-(D43-0.5)*hl/10</f>
         <v>87.021126760563376</v>
       </c>
@@ -1639,20 +1846,20 @@
         <f>fy/gammaM*(1-C43*(1-ka)/hl)</f>
         <v>338.96250832236842</v>
       </c>
-      <c r="H43" s="22">
+      <c r="H43" s="23">
         <f t="shared" si="1"/>
         <v>21.735612787184213</v>
       </c>
-      <c r="I43" s="21">
+      <c r="I43" s="22">
         <f t="shared" si="2"/>
-        <v>4916.4520935564151</v>
-      </c>
-      <c r="J43" s="21">
+        <v>4974.1444012487227</v>
+      </c>
+      <c r="J43" s="22">
         <f t="shared" si="0"/>
         <v>268.81669849408019</v>
       </c>
     </row>
-    <row r="44" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C44" s="12">
         <f>(hl/10)*(D44-0.5)</f>
         <v>11.450704225352112</v>
@@ -1660,11 +1867,11 @@
       <c r="D44" s="3">
         <v>2</v>
       </c>
-      <c r="E44" s="20">
+      <c r="E44" s="21">
         <f>E43</f>
         <v>64.123943661971836</v>
       </c>
-      <c r="F44" s="20">
+      <c r="F44" s="21">
         <f>Tf+hl-(D44-0.5)*hl/10</f>
         <v>79.387323943661968</v>
       </c>
@@ -1672,29 +1879,29 @@
         <f>fy/gammaM*(1-C44*(1-ka)/hl)</f>
         <v>306.88752496710526</v>
       </c>
-      <c r="H44" s="22">
+      <c r="H44" s="23">
         <f t="shared" si="1"/>
         <v>19.678838361552632</v>
       </c>
-      <c r="I44" s="21">
+      <c r="I44" s="22">
         <f t="shared" si="2"/>
-        <v>4936.1309319179682</v>
-      </c>
-      <c r="J44" s="21">
+        <v>4993.8232396102758</v>
+      </c>
+      <c r="J44" s="22">
         <f t="shared" si="0"/>
         <v>247.08108570689598</v>
       </c>
     </row>
-    <row r="45" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C45" s="12"/>
       <c r="D45" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E45" s="25">
+      <c r="E45" s="26">
         <f>nbPhi*Phi^2/4*PI()</f>
         <v>226.1946710584651</v>
       </c>
-      <c r="F45" s="25">
+      <c r="F45" s="26">
         <f>Tf+ui</f>
         <v>74.5</v>
       </c>
@@ -1702,20 +1909,20 @@
         <f>kr*fsk/GammaS</f>
         <v>197.57289979099301</v>
       </c>
-      <c r="H45" s="22">
+      <c r="H45" s="23">
         <f t="shared" si="1"/>
         <v>44.689937078290747</v>
       </c>
-      <c r="I45" s="21">
+      <c r="I45" s="22">
         <f t="shared" si="2"/>
-        <v>4980.8208689962585</v>
-      </c>
-      <c r="J45" s="21">
+        <v>5038.5131766885661</v>
+      </c>
+      <c r="J45" s="22">
         <f t="shared" si="0"/>
         <v>227.40224734534334</v>
       </c>
     </row>
-    <row r="46" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C46" s="12">
         <f>(hl/10)*(D46-0.5)</f>
         <v>19.08450704225352</v>
@@ -1723,11 +1930,11 @@
       <c r="D46" s="3">
         <v>3</v>
       </c>
-      <c r="E46" s="20">
+      <c r="E46" s="21">
         <f>E44</f>
         <v>64.123943661971836</v>
       </c>
-      <c r="F46" s="20">
+      <c r="F46" s="21">
         <f>Tf+hl-(D46-0.5)*hl/10</f>
         <v>71.75352112676056</v>
       </c>
@@ -1735,20 +1942,20 @@
         <f>fy/gammaM*(1-C46*(1-ka)/hl)</f>
         <v>274.81254161184211</v>
       </c>
-      <c r="H46" s="22">
+      <c r="H46" s="23">
         <f t="shared" si="1"/>
         <v>17.622063935921055</v>
       </c>
-      <c r="I46" s="21">
+      <c r="I46" s="22">
         <f t="shared" si="2"/>
-        <v>4998.4429329321792</v>
-      </c>
-      <c r="J46" s="21">
+        <v>5056.1352406244869</v>
+      </c>
+      <c r="J46" s="22">
         <f t="shared" si="0"/>
         <v>182.7123102670526</v>
       </c>
     </row>
-    <row r="47" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C47" s="12">
         <f>(hl/10)*(D47-0.5)</f>
         <v>26.718309859154928</v>
@@ -1756,11 +1963,11 @@
       <c r="D47" s="3">
         <v>4</v>
       </c>
-      <c r="E47" s="20">
+      <c r="E47" s="21">
         <f t="shared" ref="E47:E53" si="3">E46</f>
         <v>64.123943661971836</v>
       </c>
-      <c r="F47" s="20">
+      <c r="F47" s="21">
         <f>Tf+hl-(D47-0.5)*hl/10</f>
         <v>64.119718309859152</v>
       </c>
@@ -1768,20 +1975,20 @@
         <f>fy/gammaM*(1-C47*(1-ka)/hl)</f>
         <v>242.73755825657892</v>
       </c>
-      <c r="H47" s="22">
+      <c r="H47" s="23">
         <f t="shared" si="1"/>
         <v>15.565289510289473</v>
       </c>
-      <c r="I47" s="21">
+      <c r="I47" s="22">
         <f t="shared" si="2"/>
-        <v>5014.0082224424687</v>
-      </c>
-      <c r="J47" s="21">
+        <v>5071.7005301347763</v>
+      </c>
+      <c r="J47" s="22">
         <f t="shared" si="0"/>
         <v>165.09024633113154</v>
       </c>
     </row>
-    <row r="48" spans="2:14" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:16" x14ac:dyDescent="0.25">
       <c r="C48" s="12">
         <f>(hl/10)*(D48-0.5)</f>
         <v>34.352112676056336</v>
@@ -1789,11 +1996,11 @@
       <c r="D48" s="3">
         <v>5</v>
       </c>
-      <c r="E48" s="20">
+      <c r="E48" s="21">
         <f t="shared" si="3"/>
         <v>64.123943661971836</v>
       </c>
-      <c r="F48" s="20">
+      <c r="F48" s="21">
         <f>Tf+hl-(D48-0.5)*hl/10</f>
         <v>56.485915492957744</v>
       </c>
@@ -1801,15 +2008,15 @@
         <f>fy/gammaM*(1-C48*(1-ka)/hl)</f>
         <v>210.66257490131579</v>
       </c>
-      <c r="H48" s="22">
+      <c r="H48" s="23">
         <f t="shared" si="1"/>
         <v>13.508515084657896</v>
       </c>
-      <c r="I48" s="21">
+      <c r="I48" s="22">
         <f t="shared" si="2"/>
-        <v>5027.5167375271267</v>
-      </c>
-      <c r="J48" s="21">
+        <v>5085.2090452194343</v>
+      </c>
+      <c r="J48" s="22">
         <f t="shared" si="0"/>
         <v>149.52495682084208</v>
       </c>
@@ -1822,11 +2029,11 @@
       <c r="D49" s="3">
         <v>6</v>
       </c>
-      <c r="E49" s="20">
+      <c r="E49" s="21">
         <f t="shared" si="3"/>
         <v>64.123943661971836</v>
       </c>
-      <c r="F49" s="20">
+      <c r="F49" s="21">
         <f>Tf+hl-(D49-0.5)*hl/10</f>
         <v>48.852112676056336</v>
       </c>
@@ -1834,15 +2041,15 @@
         <f>fy/gammaM*(1-C49*(1-ka)/hl)</f>
         <v>178.58759154605261</v>
       </c>
-      <c r="H49" s="22">
+      <c r="H49" s="23">
         <f t="shared" si="1"/>
         <v>11.451740659026315</v>
       </c>
-      <c r="I49" s="21">
+      <c r="I49" s="22">
         <f t="shared" si="2"/>
-        <v>5038.9684781861533</v>
-      </c>
-      <c r="J49" s="21">
+        <v>5096.660785878461</v>
+      </c>
+      <c r="J49" s="22">
         <f t="shared" si="0"/>
         <v>136.01644173618419</v>
       </c>
@@ -1855,11 +2062,11 @@
       <c r="D50" s="3">
         <v>7</v>
       </c>
-      <c r="E50" s="20">
+      <c r="E50" s="21">
         <f t="shared" si="3"/>
         <v>64.123943661971836</v>
       </c>
-      <c r="F50" s="20">
+      <c r="F50" s="21">
         <f>Tf+hl-(D50-0.5)*hl/10</f>
         <v>41.218309859154928</v>
       </c>
@@ -1867,15 +2074,15 @@
         <f>fy/gammaM*(1-C50*(1-ka)/hl)</f>
         <v>146.51260819078948</v>
       </c>
-      <c r="H50" s="22">
+      <c r="H50" s="23">
         <f t="shared" si="1"/>
         <v>9.3949662333947384</v>
       </c>
-      <c r="I50" s="21">
+      <c r="I50" s="22">
         <f t="shared" si="2"/>
-        <v>5048.3634444195477</v>
-      </c>
-      <c r="J50" s="21">
+        <v>5106.0557521118553</v>
+      </c>
+      <c r="J50" s="22">
         <f t="shared" si="0"/>
         <v>124.56470107715788</v>
       </c>
@@ -1888,11 +2095,11 @@
       <c r="D51" s="3">
         <v>8</v>
       </c>
-      <c r="E51" s="20">
+      <c r="E51" s="21">
         <f t="shared" si="3"/>
         <v>64.123943661971836</v>
       </c>
-      <c r="F51" s="20">
+      <c r="F51" s="21">
         <f>Tf+hl-(D51-0.5)*hl/10</f>
         <v>33.58450704225352</v>
       </c>
@@ -1900,15 +2107,15 @@
         <f>fy/gammaM*(1-C51*(1-ka)/hl)</f>
         <v>114.43762483552629</v>
       </c>
-      <c r="H51" s="22">
+      <c r="H51" s="23">
         <f t="shared" si="1"/>
         <v>7.3381918077631569</v>
       </c>
-      <c r="I51" s="21">
+      <c r="I51" s="22">
         <f t="shared" si="2"/>
-        <v>5055.7016362273107</v>
-      </c>
-      <c r="J51" s="21">
+        <v>5113.3939439196183</v>
+      </c>
+      <c r="J51" s="22">
         <f t="shared" si="0"/>
         <v>115.16973484376314</v>
       </c>
@@ -1921,11 +2128,11 @@
       <c r="D52" s="3">
         <v>9</v>
       </c>
-      <c r="E52" s="20">
+      <c r="E52" s="21">
         <f t="shared" si="3"/>
         <v>64.123943661971836</v>
       </c>
-      <c r="F52" s="20">
+      <c r="F52" s="21">
         <f>Tf+hl-(D52-0.5)*hl/10</f>
         <v>25.950704225352112</v>
       </c>
@@ -1933,15 +2140,15 @@
         <f>fy/gammaM*(1-C52*(1-ka)/hl)</f>
         <v>82.36264148026315</v>
       </c>
-      <c r="H52" s="22">
+      <c r="H52" s="23">
         <f t="shared" si="1"/>
         <v>5.2814173821315791</v>
       </c>
-      <c r="I52" s="21">
+      <c r="I52" s="22">
         <f t="shared" si="2"/>
-        <v>5060.9830536094423</v>
-      </c>
-      <c r="J52" s="21">
+        <v>5118.6753613017499</v>
+      </c>
+      <c r="J52" s="22">
         <f t="shared" si="0"/>
         <v>107.83154303599999</v>
       </c>
@@ -1954,27 +2161,27 @@
       <c r="D53" s="3">
         <v>10</v>
       </c>
-      <c r="E53" s="20">
+      <c r="E53" s="21">
         <f t="shared" si="3"/>
         <v>64.123943661971836</v>
       </c>
-      <c r="F53" s="20">
+      <c r="F53" s="21">
         <f>Tf+hl-(D53-0.5)*hl/10</f>
         <v>18.316901408450704</v>
       </c>
-      <c r="G53" s="28">
+      <c r="G53" s="29">
         <f>fy/gammaM*(1-C53*(1-ka)/hl)</f>
         <v>50.287658124999972</v>
       </c>
-      <c r="H53" s="24">
+      <c r="H53" s="25">
         <f t="shared" si="1"/>
         <v>3.2246429564999985</v>
       </c>
-      <c r="I53" s="21">
+      <c r="I53" s="22">
         <f t="shared" si="2"/>
-        <v>5064.2076965659426</v>
-      </c>
-      <c r="J53" s="21">
+        <v>5121.9000042582502</v>
+      </c>
+      <c r="J53" s="22">
         <f>J54+H53</f>
         <v>102.55012565386841</v>
       </c>
@@ -1983,7 +2190,7 @@
       <c r="D54" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E54" s="19">
+      <c r="E54" s="20">
         <f>bf*Tf</f>
         <v>2900</v>
       </c>
@@ -1995,15 +2202,15 @@
         <f>ka*fy/gammaM</f>
         <v>34.250166447368414</v>
       </c>
-      <c r="H54" s="19">
+      <c r="H54" s="20">
         <f t="shared" si="1"/>
         <v>99.3254826973684</v>
       </c>
-      <c r="I54" s="21">
+      <c r="I54" s="22">
         <f t="shared" si="2"/>
-        <v>5163.5331792633106</v>
-      </c>
-      <c r="J54" s="21">
+        <v>5221.2254869556182</v>
+      </c>
+      <c r="J54" s="22">
         <f>H54</f>
         <v>99.3254826973684</v>
       </c>
@@ -2019,7 +2226,7 @@
       </c>
       <c r="E59" s="16">
         <f>(SUM(H40:H54)/H38)</f>
-        <v>0.70786748576269387</v>
+        <v>0.69425464949802673</v>
       </c>
     </row>
     <row r="60" spans="3:13" x14ac:dyDescent="0.25">
@@ -2028,7 +2235,7 @@
       </c>
       <c r="E60" s="17">
         <f>p*hch</f>
-        <v>36.101241773897385</v>
+        <v>36.101241773897392</v>
       </c>
       <c r="F60" t="s">
         <v>4</v>
@@ -2045,6 +2252,13 @@
       <c r="F61" t="s">
         <v>4</v>
       </c>
+      <c r="H61" s="18">
+        <f>zANP-Ht</f>
+        <v>103.89875822610259</v>
+      </c>
+      <c r="I61" t="s">
+        <v>4</v>
+      </c>
     </row>
     <row r="64" spans="3:13" x14ac:dyDescent="0.25">
       <c r="E64" s="5" t="s">
@@ -2059,7 +2273,7 @@
       <c r="H64" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="I64" s="26" t="s">
+      <c r="I64" s="27" t="s">
         <v>74</v>
       </c>
       <c r="M64">
@@ -2068,19 +2282,19 @@
       </c>
     </row>
     <row r="65" spans="4:20" x14ac:dyDescent="0.25">
-      <c r="E65" s="18" t="s">
+      <c r="E65" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="F65" s="18" t="s">
+      <c r="F65" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="G65" s="18" t="s">
+      <c r="G65" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="H65" s="18" t="s">
+      <c r="H65" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="I65" s="18" t="s">
+      <c r="I65" s="19" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2088,11 +2302,11 @@
       <c r="D66" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="E66" s="19">
+      <c r="E66" s="20">
         <f>beff*1000*tcp</f>
-        <v>90253.104434743465</v>
-      </c>
-      <c r="F66" s="19">
+        <v>90253.10443474348</v>
+      </c>
+      <c r="F66" s="20">
         <f>Ht+Td-tcp/2</f>
         <v>618.94937911305135</v>
       </c>
@@ -2100,25 +2314,25 @@
         <f>fck/GammaC</f>
         <v>23.076923076923077</v>
       </c>
-      <c r="H66" s="19">
+      <c r="H66" s="20">
         <f>G66*E66/1000</f>
         <v>2082.7639484940801</v>
       </c>
-      <c r="I66" s="20">
+      <c r="I66" s="21">
         <f>H66*ABS(F66-zANP)/1000</f>
         <v>37.59518243127112</v>
       </c>
-      <c r="K66" s="19">
+      <c r="K66" s="20">
         <f>(Ht+Td-F66)</f>
         <v>18.05062088694865</v>
       </c>
-      <c r="R66" s="20">
+      <c r="R66" s="21">
         <v>2082</v>
       </c>
-      <c r="S66" s="20">
+      <c r="S66" s="21">
         <v>36.1</v>
       </c>
-      <c r="T66" s="20">
+      <c r="T66" s="21">
         <f>R66*S66/2000</f>
         <v>37.580100000000002</v>
       </c>
@@ -2127,28 +2341,28 @@
       <c r="D67" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="E67" s="19">
+      <c r="E67" s="20">
         <v>0</v>
       </c>
-      <c r="F67" s="19">
+      <c r="F67" s="20">
         <v>1</v>
       </c>
-      <c r="G67" s="19">
+      <c r="G67" s="20">
         <v>2</v>
       </c>
-      <c r="H67" s="19">
+      <c r="H67" s="20">
         <f t="shared" ref="H67:H73" si="4">G67*E67/1000</f>
         <v>0</v>
       </c>
-      <c r="I67" s="20">
+      <c r="I67" s="21">
         <f>H67*ABS(F67-zANP)/1000</f>
         <v>0</v>
       </c>
-      <c r="K67" s="19">
+      <c r="K67" s="20">
         <f>(Ht+Td-F67)</f>
         <v>636</v>
       </c>
-      <c r="R67" s="20">
+      <c r="R67" s="21">
         <v>0</v>
       </c>
     </row>
@@ -2156,31 +2370,31 @@
       <c r="D68" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="E68" s="19">
+      <c r="E68" s="20">
         <f>E40</f>
         <v>1819.75</v>
       </c>
-      <c r="F68" s="19">
+      <c r="F68" s="20">
         <f t="shared" ref="F68:G68" si="5">F40</f>
         <v>489.75</v>
       </c>
-      <c r="G68" s="19">
+      <c r="G68" s="20">
         <f t="shared" si="5"/>
         <v>355</v>
       </c>
-      <c r="H68" s="19">
+      <c r="H68" s="20">
         <f t="shared" si="4"/>
         <v>646.01125000000002</v>
       </c>
-      <c r="I68" s="20">
+      <c r="I68" s="21">
         <f>H68*ABS(F68-zANP)/1000</f>
         <v>71.803348237592317</v>
       </c>
-      <c r="K68" s="19">
+      <c r="K68" s="20">
         <f>(Ht+Td-F68)</f>
         <v>147.25</v>
       </c>
-      <c r="R68" s="29">
+      <c r="R68" s="30">
         <v>646</v>
       </c>
       <c r="S68" s="5">
@@ -2195,27 +2409,27 @@
       <c r="D69" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E69" s="19">
+      <c r="E69" s="20">
         <f t="shared" ref="E69:G70" si="6">E41</f>
         <v>0</v>
       </c>
-      <c r="F69" s="19">
+      <c r="F69" s="20">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="G69" s="19">
+      <c r="G69" s="20">
         <f t="shared" si="6"/>
         <v>355</v>
       </c>
-      <c r="H69" s="19">
+      <c r="H69" s="20">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="I69" s="20">
+      <c r="I69" s="21">
         <f>H69*ABS(F69-zANP)/1000</f>
         <v>0</v>
       </c>
-      <c r="K69" s="19">
+      <c r="K69" s="20">
         <f>(Ht+Td-F69)</f>
         <v>637</v>
       </c>
@@ -2225,27 +2439,27 @@
       <c r="D70" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="E70" s="19">
+      <c r="E70" s="20">
         <f t="shared" si="6"/>
         <v>3289.9605633802817</v>
       </c>
-      <c r="F70" s="19">
+      <c r="F70" s="20">
         <f t="shared" si="6"/>
         <v>286.66901408450701</v>
       </c>
-      <c r="G70" s="19">
+      <c r="G70" s="20">
         <f t="shared" si="6"/>
         <v>355</v>
       </c>
-      <c r="H70" s="19">
+      <c r="H70" s="20">
         <f t="shared" si="4"/>
         <v>1167.9359999999999</v>
       </c>
-      <c r="I70" s="20">
+      <c r="I70" s="21">
         <f>H70*ABS(F70-zANP)/1000</f>
         <v>367.00023045375855</v>
       </c>
-      <c r="K70" s="19">
+      <c r="K70" s="20">
         <f>(Ht+Td-F70)</f>
         <v>350.33098591549299</v>
       </c>
@@ -2258,10 +2472,10 @@
       <c r="O70" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="P70" s="26" t="s">
+      <c r="P70" s="27" t="s">
         <v>77</v>
       </c>
-      <c r="R70" s="29">
+      <c r="R70" s="30">
         <v>1168</v>
       </c>
       <c r="S70" s="5">
@@ -2276,34 +2490,34 @@
       <c r="D71" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="E71" s="19">
+      <c r="E71" s="20">
         <f>hl*Tw</f>
         <v>641.23943661971828</v>
       </c>
-      <c r="F71" s="19">
+      <c r="F71" s="20">
         <f>Tf+M73</f>
         <v>63.334098184427475</v>
       </c>
-      <c r="G71" s="19">
+      <c r="G71" s="20">
         <f>AVERAGE(G70,G72)</f>
         <v>194.62508322368421</v>
       </c>
-      <c r="H71" s="19">
+      <c r="H71" s="20">
         <f t="shared" si="4"/>
         <v>124.80127871842105</v>
       </c>
-      <c r="I71" s="20">
+      <c r="I71" s="21">
         <f>H71*ABS(F71-zANP)/1000</f>
         <v>67.088756967034357</v>
       </c>
-      <c r="K71" s="19">
+      <c r="K71" s="20">
         <f>(Ht+Td-F71)</f>
         <v>573.66590181557251</v>
       </c>
       <c r="L71">
         <v>1</v>
       </c>
-      <c r="M71" s="20">
+      <c r="M71" s="21">
         <f>hl/2</f>
         <v>38.16901408450704</v>
       </c>
@@ -2311,7 +2525,7 @@
         <f>ka*fy/gammaM</f>
         <v>34.250166447368414</v>
       </c>
-      <c r="O71" s="20">
+      <c r="O71" s="21">
         <f>hl*Tw*N71/1000</f>
         <v>21.962557436842101</v>
       </c>
@@ -2319,7 +2533,7 @@
         <f>O71*M71</f>
         <v>838.289164138621</v>
       </c>
-      <c r="R71" s="29">
+      <c r="R71" s="30">
         <v>124.7</v>
       </c>
       <c r="S71" s="5">
@@ -2334,34 +2548,34 @@
       <c r="D72" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E72" s="19">
+      <c r="E72" s="20">
         <f>E54</f>
         <v>2900</v>
       </c>
-      <c r="F72" s="19">
+      <c r="F72" s="20">
         <f>F54</f>
         <v>7.25</v>
       </c>
-      <c r="G72" s="19">
+      <c r="G72" s="20">
         <f>G54</f>
         <v>34.250166447368414</v>
       </c>
-      <c r="H72" s="19">
+      <c r="H72" s="20">
         <f t="shared" si="4"/>
         <v>99.3254826973684</v>
       </c>
-      <c r="I72" s="20">
+      <c r="I72" s="21">
         <f>H72*ABS(F72-zANP)/1000</f>
         <v>58.964449463500991</v>
       </c>
-      <c r="K72" s="19">
+      <c r="K72" s="20">
         <f>(Ht+Td-F72)</f>
         <v>629.75</v>
       </c>
       <c r="L72">
         <v>2</v>
       </c>
-      <c r="M72" s="20">
+      <c r="M72" s="21">
         <f>2*hl/3</f>
         <v>50.89201877934272</v>
       </c>
@@ -2369,7 +2583,7 @@
         <f>fy/gammaM</f>
         <v>355</v>
       </c>
-      <c r="O72" s="20">
+      <c r="O72" s="21">
         <f>hl*Tw*N72/1000/2</f>
         <v>113.82</v>
       </c>
@@ -2377,7 +2591,7 @@
         <f>O72*M72</f>
         <v>5792.5295774647884</v>
       </c>
-      <c r="R72" s="29">
+      <c r="R72" s="30">
         <v>99.346999999999994</v>
       </c>
       <c r="S72" s="5">
@@ -2392,15 +2606,15 @@
       <c r="D73" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="E73" s="19">
+      <c r="E73" s="20">
         <f>E45</f>
         <v>226.1946710584651</v>
       </c>
-      <c r="F73" s="19">
+      <c r="F73" s="20">
         <f t="shared" ref="F73:G73" si="8">F45</f>
         <v>74.5</v>
       </c>
-      <c r="G73" s="19">
+      <c r="G73" s="20">
         <f t="shared" si="8"/>
         <v>197.57289979099301</v>
       </c>
@@ -2408,22 +2622,22 @@
         <f t="shared" si="4"/>
         <v>44.689937078290747</v>
       </c>
-      <c r="I73" s="20">
+      <c r="I73" s="21">
         <f>H73*ABS(F73-zANP)/1000</f>
         <v>23.524727383214909</v>
       </c>
-      <c r="K73" s="19">
+      <c r="K73" s="20">
         <f>(Ht+Td-F73)</f>
         <v>562.5</v>
       </c>
       <c r="L73" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="M73" s="20">
+      <c r="M73" s="21">
         <f>SUM(P71:P72)/SUM(O71:O72)</f>
         <v>48.834098184427475</v>
       </c>
-      <c r="R73" s="29">
+      <c r="R73" s="30">
         <v>44.6</v>
       </c>
       <c r="S73" s="5">
@@ -2435,7 +2649,7 @@
       </c>
     </row>
     <row r="75" spans="4:20" x14ac:dyDescent="0.25">
-      <c r="I75" s="27">
+      <c r="I75" s="28">
         <f>SUM(I66:I73)</f>
         <v>625.97669493637216</v>
       </c>
@@ -2445,6 +2659,21 @@
       <c r="T75" s="12">
         <f>SUM(T66:T73)</f>
         <v>626.58746105</v>
+      </c>
+    </row>
+    <row r="80" spans="4:20" x14ac:dyDescent="0.25">
+      <c r="D80" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E80" s="4">
+        <f>Ht-Tf-ui</f>
+        <v>422.5</v>
+      </c>
+    </row>
+    <row r="81" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E81">
+        <f>461-E80</f>
+        <v>38.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>